<commit_message>
docs(qms): Excel registers EM26-19…22 approved (AR-2026-003)
Alexander Peter (review), Sheryl Nazareth (QA) and Anita Johan (Managing Director)
confirmed the four registers on 2026-10-12. Approval record:
docs/qms/records/approvals/2026-10-12_AR-2026-003_register_approval.md

- EM26-19…22: status APPROVED, signatures dated 2026-10-12
- Also reviewed with them: gap analysis 8.2 / 9.1.2 re-rating, REG-01 entries, evidence README
- REG-01, QM-01 and the README point to AR-2026-003

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qms/evidence-2026/19_Excel_Registers/EM26-19_Deliverable_Review_Feedback_and_Action_Log.xlsx
+++ b/docs/qms/evidence-2026/19_Excel_Registers/EM26-19_Deliverable_Review_Feedback_and_Action_Log.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -646,7 +646,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Issued 2026-10-11 for review and approval</t>
+          <t>APPROVED — 2026-10-12 (AR-2026-003)</t>
         </is>
       </c>
       <c r="C11" s="2" t="n"/>
@@ -847,10 +847,14 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>To be confirmed</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr"/>
+          <t>Alexander Peter</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -865,10 +869,14 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>To be confirmed</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr"/>
+          <t>Sheryl Nazareth</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -883,10 +891,14 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>To be confirmed</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr"/>
+          <t>Anita Johan</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n"/>
@@ -897,44 +909,92 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Version</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Change</t>
-        </is>
-      </c>
+          <t>Approval record</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
+          <t>docs/qms/records/approvals/2026-10-12_AR-2026-003_register_approval.md — review and approval confirmed by each role holder on 2026-10-12. Signatures are their typed names (SOP-01 §6).</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
           <t>2026-10-11</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>Richard Watson Stephen Amudha (Lead Engineer)</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>First issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Anita Johan (Managing Director)</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Approved — AR-2026-003</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1455,7 @@
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(qms): revision 1.1 of the Excel registers approved (AR-2026-004) — versions v1.0.0 → v1.4.1
Alexander Peter (review), Sheryl Nazareth (QA) and Anita Johan (Managing Director)
confirmed revision 1.1 on 2026-10-12. Approval record:
docs/qms/records/approvals/2026-10-12_AR-2026-004_register_revision_approval.md

- EM26-19…22 rev 1.1: status APPROVED, signatures dated 2026-10-12
- REG-01, QM-01 and the evidence README point to AR-2026-004

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qms/evidence-2026/19_Excel_Registers/EM26-19_Deliverable_Review_Feedback_and_Action_Log.xlsx
+++ b/docs/qms/evidence-2026/19_Excel_Registers/EM26-19_Deliverable_Review_Feedback_and_Action_Log.xlsx
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -647,7 +647,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Rev 1.0 APPROVED 2026-10-12 (AR-2026-003); rev 1.1 issued 2026-10-12 — approval of the revision to be confirmed</t>
+          <t>APPROVED — rev 1.1 2026-10-12 (AR-2026-004); rev 1.0 2026-10-12 (AR-2026-003)</t>
         </is>
       </c>
       <c r="C11" s="2" t="n"/>
@@ -862,10 +862,14 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Rev 1.0 signed 2026-10-12; rev 1.1 to confirm</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr"/>
+          <t>Alexander Peter</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -880,10 +884,14 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Rev 1.0 signed 2026-10-12; rev 1.1 to confirm</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr"/>
+          <t>Sheryl Nazareth</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -898,10 +906,14 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Rev 1.0 signed 2026-10-12; rev 1.1 to confirm</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr"/>
+          <t>Anita Johan</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n"/>
@@ -922,7 +934,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Rev 1.0: docs/qms/records/approvals/2026-10-12_AR-2026-003_register_approval.md — confirmed by each role holder on 2026-10-12. Rev 1.1 is signed here when they confirm it. Signatures are their typed names (SOP-01 §6).</t>
+          <t>Rev 1.1: docs/qms/records/approvals/2026-10-12_AR-2026-004_register_revision_approval.md; rev 1.0: …/2026-10-12_AR-2026-003_register_approval.md. Review and approval confirmed by each role holder; signatures are their typed names (SOP-01 §6).</t>
         </is>
       </c>
       <c r="B31" s="2" t="n"/>
@@ -1020,6 +1032,28 @@
       <c r="D36" s="5" t="inlineStr">
         <is>
           <t>Versions v1.0.0–v1.4.1 added (v1.0.0–v1.3.0 retrospective baselines, REG-08 §2a); version reviews</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Anita Johan (Managing Director)</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Approved — AR-2026-004</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1514,7 @@
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>

</xml_diff>